<commit_message>
updates data prep script
</commit_message>
<xml_diff>
--- a/docs/cols_hbsc2018 v2 definitive.xlsx
+++ b/docs/cols_hbsc2018 v2 definitive.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MisLocalFiles\Github\HBSC\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{211B41C6-2EC3-4CD6-B980-56593408BC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF4756F-6E2D-4521-8371-8B817F14D3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="22560" windowHeight="13440" xr2:uid="{ECC3AB54-F37C-492C-8A31-6024B29491CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECC3AB54-F37C-492C-8A31-6024B29491CE}"/>
   </bookViews>
   <sheets>
     <sheet name="hbsc2018_cols (2)" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="177">
   <si>
     <t>HBSC</t>
   </si>
@@ -439,27 +439,12 @@
     <t>family support</t>
   </si>
   <si>
-    <t>My family really
-tries to help me</t>
-  </si>
-  <si>
     <t>values</t>
   </si>
   <si>
     <t>1-7 likert</t>
   </si>
   <si>
-    <t>I get the emotional
-help and support I
-need from my
-family</t>
-  </si>
-  <si>
-    <t>I can talk about
-my problems with
-my family</t>
-  </si>
-  <si>
     <t>family affluence</t>
   </si>
   <si>
@@ -515,13 +500,73 @@
   </si>
   <si>
     <t>1 excellent to 4 poor</t>
+  </si>
+  <si>
+    <t>help make decisiones</t>
+  </si>
+  <si>
+    <t>tries to help me</t>
+  </si>
+  <si>
+    <t>give me emotional support</t>
+  </si>
+  <si>
+    <t>I can talk problems</t>
+  </si>
+  <si>
+    <t>peer support</t>
+  </si>
+  <si>
+    <t>try to help</t>
+  </si>
+  <si>
+    <t>can count on</t>
+  </si>
+  <si>
+    <t>I can share</t>
+  </si>
+  <si>
+    <t>1-7</t>
+  </si>
+  <si>
+    <t>1-8</t>
+  </si>
+  <si>
+    <t>1-9</t>
+  </si>
+  <si>
+    <t>1-10</t>
+  </si>
+  <si>
+    <t>teacher support</t>
+  </si>
+  <si>
+    <t>accepts me</t>
+  </si>
+  <si>
+    <t>cares about me</t>
+  </si>
+  <si>
+    <t>I trust him</t>
+  </si>
+  <si>
+    <t>1-5</t>
+  </si>
+  <si>
+    <t>classmate support</t>
+  </si>
+  <si>
+    <t>we like be together</t>
+  </si>
+  <si>
+    <t>me ayudan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -656,8 +701,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -858,6 +909,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1022,7 +1091,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1046,6 +1115,21 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1424,16 +1508,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAAD171-0304-433A-92B8-84371DC226A9}">
   <dimension ref="A1:D121"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.81640625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7109375" style="2"/>
+    <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>120</v>
       </c>
@@ -1444,135 +1528,135 @@
         <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>25</v>
       </c>
@@ -1580,13 +1664,13 @@
         <v>25</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>26</v>
       </c>
@@ -1600,379 +1684,469 @@
         <v>134</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C29" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C30" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C31" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C32" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C33" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C34" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C35" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C36" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C47" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="12" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
+      <c r="B60" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="12" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
+      <c r="B61" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="12" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
+      <c r="B62" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="10" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" s="2" t="s">
+      <c r="B63" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="10" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="2" t="s">
+      <c r="B64" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="10" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B65" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="2" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" s="6" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="2" t="s">
+      <c r="B72" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" s="6" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="2" t="s">
+      <c r="B73" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="6" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="2" t="s">
+      <c r="B74" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B75" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>74</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>75</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>76</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>77</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A83" s="4" t="s">
         <v>81</v>
       </c>
@@ -1983,10 +2157,10 @@
         <v>124</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="s">
         <v>82</v>
       </c>
@@ -1997,10 +2171,10 @@
         <v>125</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="4" t="s">
         <v>83</v>
       </c>
@@ -2011,10 +2185,10 @@
         <v>126</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="4" t="s">
         <v>84</v>
       </c>
@@ -2025,10 +2199,10 @@
         <v>127</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A87" s="4" t="s">
         <v>85</v>
       </c>
@@ -2039,10 +2213,10 @@
         <v>128</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="4" t="s">
         <v>86</v>
       </c>
@@ -2053,10 +2227,10 @@
         <v>129</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A89" s="4" t="s">
         <v>87</v>
       </c>
@@ -2067,10 +2241,10 @@
         <v>130</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="4" t="s">
         <v>88</v>
       </c>
@@ -2081,10 +2255,10 @@
         <v>131</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="4" t="s">
         <v>89</v>
       </c>
@@ -2095,121 +2269,121 @@
         <v>132</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>107</v>
       </c>
       <c r="B109" s="7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>108</v>
       </c>
       <c r="B110" s="7"/>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>109</v>
       </c>
       <c r="B111" s="7"/>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>110</v>
       </c>
       <c r="B112" s="7"/>
     </row>
-    <row r="113" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>111</v>
       </c>
@@ -2217,13 +2391,13 @@
         <v>135</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
         <v>112</v>
       </c>
@@ -2231,13 +2405,13 @@
         <v>135</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
         <v>113</v>
       </c>
@@ -2245,61 +2419,71 @@
         <v>135</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" s="5" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B116" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="6" t="s">
         <v>116</v>
       </c>
       <c r="B118" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C118" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="D118" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="6" t="s">
         <v>117</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>119</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2307,17 +2491,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595DF94D-C0B1-43ED-A269-37084843006E}">
   <dimension ref="A1:B121"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B1">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2325,7 +2509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2333,7 +2517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2341,7 +2525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2349,7 +2533,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2357,7 +2541,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2365,7 +2549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -2373,7 +2557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2381,7 +2565,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2389,7 +2573,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2397,7 +2581,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2405,7 +2589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2413,7 +2597,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2421,7 +2605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2429,7 +2613,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2437,7 +2621,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2445,7 +2629,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2453,7 +2637,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2461,7 +2645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -2469,7 +2653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2477,7 +2661,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -2485,7 +2669,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2493,7 +2677,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -2501,7 +2685,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -2509,7 +2693,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -2517,7 +2701,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -2525,7 +2709,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -2533,7 +2717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -2541,7 +2725,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -2549,7 +2733,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -2557,7 +2741,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -2565,7 +2749,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -2573,7 +2757,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -2581,7 +2765,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -2589,7 +2773,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -2597,7 +2781,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -2605,7 +2789,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -2613,7 +2797,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -2621,7 +2805,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -2629,7 +2813,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -2637,7 +2821,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -2645,7 +2829,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -2653,7 +2837,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -2661,7 +2845,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -2669,7 +2853,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -2677,7 +2861,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -2685,7 +2869,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>46</v>
       </c>
@@ -2693,7 +2877,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -2701,7 +2885,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -2709,7 +2893,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -2717,7 +2901,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -2725,7 +2909,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -2733,7 +2917,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>52</v>
       </c>
@@ -2741,7 +2925,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -2749,7 +2933,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -2757,7 +2941,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>55</v>
       </c>
@@ -2765,7 +2949,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>56</v>
       </c>
@@ -2773,7 +2957,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>57</v>
       </c>
@@ -2781,7 +2965,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -2789,7 +2973,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>59</v>
       </c>
@@ -2797,7 +2981,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>60</v>
       </c>
@@ -2805,7 +2989,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>61</v>
       </c>
@@ -2813,7 +2997,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>62</v>
       </c>
@@ -2821,7 +3005,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -2829,7 +3013,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -2837,7 +3021,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>65</v>
       </c>
@@ -2845,7 +3029,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>66</v>
       </c>
@@ -2853,7 +3037,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -2861,7 +3045,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>68</v>
       </c>
@@ -2869,7 +3053,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>69</v>
       </c>
@@ -2877,7 +3061,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -2885,7 +3069,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -2893,7 +3077,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>72</v>
       </c>
@@ -2901,7 +3085,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -2909,7 +3093,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>74</v>
       </c>
@@ -2917,7 +3101,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>75</v>
       </c>
@@ -2925,7 +3109,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>76</v>
       </c>
@@ -2933,7 +3117,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>77</v>
       </c>
@@ -2941,7 +3125,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -2949,7 +3133,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>79</v>
       </c>
@@ -2957,7 +3141,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>80</v>
       </c>
@@ -2965,7 +3149,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>81</v>
       </c>
@@ -2973,7 +3157,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>82</v>
       </c>
@@ -2981,7 +3165,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -2989,7 +3173,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>84</v>
       </c>
@@ -2997,7 +3181,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>85</v>
       </c>
@@ -3005,7 +3189,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>86</v>
       </c>
@@ -3013,7 +3197,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>87</v>
       </c>
@@ -3021,7 +3205,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>88</v>
       </c>
@@ -3029,7 +3213,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>89</v>
       </c>
@@ -3037,7 +3221,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>90</v>
       </c>
@@ -3045,7 +3229,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>91</v>
       </c>
@@ -3053,7 +3237,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>92</v>
       </c>
@@ -3061,7 +3245,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>93</v>
       </c>
@@ -3069,7 +3253,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>94</v>
       </c>
@@ -3077,7 +3261,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>95</v>
       </c>
@@ -3085,7 +3269,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>96</v>
       </c>
@@ -3093,7 +3277,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>97</v>
       </c>
@@ -3101,7 +3285,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>98</v>
       </c>
@@ -3109,7 +3293,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>99</v>
       </c>
@@ -3117,7 +3301,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>100</v>
       </c>
@@ -3125,7 +3309,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>101</v>
       </c>
@@ -3133,7 +3317,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>102</v>
       </c>
@@ -3141,7 +3325,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>103</v>
       </c>
@@ -3149,7 +3333,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>104</v>
       </c>
@@ -3157,7 +3341,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>105</v>
       </c>
@@ -3165,7 +3349,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>106</v>
       </c>
@@ -3173,7 +3357,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>107</v>
       </c>
@@ -3181,7 +3365,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>108</v>
       </c>
@@ -3189,7 +3373,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>109</v>
       </c>
@@ -3197,7 +3381,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>110</v>
       </c>
@@ -3205,7 +3389,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>111</v>
       </c>
@@ -3213,7 +3397,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>112</v>
       </c>
@@ -3221,7 +3405,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>113</v>
       </c>
@@ -3229,7 +3413,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>114</v>
       </c>
@@ -3237,7 +3421,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>115</v>
       </c>
@@ -3245,7 +3429,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>116</v>
       </c>
@@ -3253,7 +3437,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>117</v>
       </c>
@@ -3261,7 +3445,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>118</v>
       </c>
@@ -3269,7 +3453,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>119</v>
       </c>

</xml_diff>